<commit_message>
Configure production release signing, fix Appium fallback execution and synchronize database task columns for Android and Web compatibilities
</commit_message>
<xml_diff>
--- a/selenium-tests/test-report.xlsx
+++ b/selenium-tests/test-report.xlsx
@@ -21,13 +21,13 @@
     <t>Report Date:</t>
   </si>
   <si>
-    <t>21/6/2026, 7:54:39 pm</t>
+    <t>22/6/2026, 11:38:17 am</t>
   </si>
   <si>
     <t>Total Duration:</t>
   </si>
   <si>
-    <t>112.75 seconds</t>
+    <t>129.43 seconds</t>
   </si>
   <si>
     <t/>
@@ -2579,7 +2579,7 @@
         <v>24</v>
       </c>
       <c r="F2" s="9">
-        <v>2828</v>
+        <v>5044</v>
       </c>
       <c r="G2" s="9" t="s">
         <v>25</v>
@@ -2602,7 +2602,7 @@
         <v>24</v>
       </c>
       <c r="F3" s="9">
-        <v>1666</v>
+        <v>2569</v>
       </c>
       <c r="G3" s="9" t="s">
         <v>25</v>
@@ -2625,7 +2625,7 @@
         <v>24</v>
       </c>
       <c r="F4" s="9">
-        <v>1310</v>
+        <v>1482</v>
       </c>
       <c r="G4" s="9" t="s">
         <v>25</v>
@@ -2648,7 +2648,7 @@
         <v>24</v>
       </c>
       <c r="F5" s="9">
-        <v>306</v>
+        <v>301</v>
       </c>
       <c r="G5" s="9" t="s">
         <v>25</v>
@@ -2671,7 +2671,7 @@
         <v>24</v>
       </c>
       <c r="F6" s="9">
-        <v>898</v>
+        <v>863</v>
       </c>
       <c r="G6" s="9" t="s">
         <v>25</v>
@@ -2694,7 +2694,7 @@
         <v>24</v>
       </c>
       <c r="F7" s="9">
-        <v>790</v>
+        <v>775</v>
       </c>
       <c r="G7" s="9" t="s">
         <v>25</v>
@@ -2717,7 +2717,7 @@
         <v>24</v>
       </c>
       <c r="F8" s="9">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="G8" s="9" t="s">
         <v>25</v>
@@ -2740,7 +2740,7 @@
         <v>24</v>
       </c>
       <c r="F9" s="9">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="G9" s="9" t="s">
         <v>25</v>
@@ -2763,7 +2763,7 @@
         <v>24</v>
       </c>
       <c r="F10" s="9">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="G10" s="9" t="s">
         <v>25</v>
@@ -2786,7 +2786,7 @@
         <v>24</v>
       </c>
       <c r="F11" s="9">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="G11" s="9" t="s">
         <v>25</v>
@@ -2809,7 +2809,7 @@
         <v>24</v>
       </c>
       <c r="F12" s="9">
-        <v>736</v>
+        <v>772</v>
       </c>
       <c r="G12" s="9" t="s">
         <v>25</v>
@@ -2832,7 +2832,7 @@
         <v>24</v>
       </c>
       <c r="F13" s="9">
-        <v>184</v>
+        <v>201</v>
       </c>
       <c r="G13" s="9" t="s">
         <v>25</v>
@@ -2855,7 +2855,7 @@
         <v>24</v>
       </c>
       <c r="F14" s="9">
-        <v>720</v>
+        <v>927</v>
       </c>
       <c r="G14" s="9" t="s">
         <v>25</v>
@@ -2878,7 +2878,7 @@
         <v>24</v>
       </c>
       <c r="F15" s="9">
-        <v>738</v>
+        <v>981</v>
       </c>
       <c r="G15" s="9" t="s">
         <v>25</v>
@@ -2901,7 +2901,7 @@
         <v>24</v>
       </c>
       <c r="F16" s="9">
-        <v>44</v>
+        <v>32</v>
       </c>
       <c r="G16" s="9" t="s">
         <v>25</v>
@@ -2924,7 +2924,7 @@
         <v>24</v>
       </c>
       <c r="F17" s="9">
-        <v>88</v>
+        <v>114</v>
       </c>
       <c r="G17" s="9" t="s">
         <v>25</v>
@@ -2947,7 +2947,7 @@
         <v>24</v>
       </c>
       <c r="F18" s="9">
-        <v>669</v>
+        <v>461</v>
       </c>
       <c r="G18" s="9" t="s">
         <v>25</v>
@@ -2970,7 +2970,7 @@
         <v>24</v>
       </c>
       <c r="F19" s="9">
-        <v>745</v>
+        <v>568</v>
       </c>
       <c r="G19" s="9" t="s">
         <v>25</v>
@@ -2993,7 +2993,7 @@
         <v>24</v>
       </c>
       <c r="F20" s="9">
-        <v>154</v>
+        <v>397</v>
       </c>
       <c r="G20" s="9" t="s">
         <v>25</v>
@@ -3016,7 +3016,7 @@
         <v>24</v>
       </c>
       <c r="F21" s="9">
-        <v>590</v>
+        <v>1259</v>
       </c>
       <c r="G21" s="9" t="s">
         <v>25</v>
@@ -3039,7 +3039,7 @@
         <v>24</v>
       </c>
       <c r="F22" s="9">
-        <v>1189</v>
+        <v>954</v>
       </c>
       <c r="G22" s="9" t="s">
         <v>25</v>
@@ -3062,7 +3062,7 @@
         <v>24</v>
       </c>
       <c r="F23" s="9">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="G23" s="9" t="s">
         <v>25</v>
@@ -3085,7 +3085,7 @@
         <v>24</v>
       </c>
       <c r="F24" s="9">
-        <v>83</v>
+        <v>112</v>
       </c>
       <c r="G24" s="9" t="s">
         <v>25</v>
@@ -3108,7 +3108,7 @@
         <v>24</v>
       </c>
       <c r="F25" s="9">
-        <v>879</v>
+        <v>448</v>
       </c>
       <c r="G25" s="9" t="s">
         <v>25</v>
@@ -3131,7 +3131,7 @@
         <v>24</v>
       </c>
       <c r="F26" s="9">
-        <v>747</v>
+        <v>775</v>
       </c>
       <c r="G26" s="9" t="s">
         <v>25</v>
@@ -3154,7 +3154,7 @@
         <v>24</v>
       </c>
       <c r="F27" s="9">
-        <v>1227</v>
+        <v>1243</v>
       </c>
       <c r="G27" s="9" t="s">
         <v>25</v>
@@ -3177,7 +3177,7 @@
         <v>24</v>
       </c>
       <c r="F28" s="9">
-        <v>1291</v>
+        <v>1213</v>
       </c>
       <c r="G28" s="9" t="s">
         <v>25</v>
@@ -3200,7 +3200,7 @@
         <v>24</v>
       </c>
       <c r="F29" s="9">
-        <v>1316</v>
+        <v>1195</v>
       </c>
       <c r="G29" s="9" t="s">
         <v>25</v>
@@ -3223,7 +3223,7 @@
         <v>24</v>
       </c>
       <c r="F30" s="9">
-        <v>781</v>
+        <v>768</v>
       </c>
       <c r="G30" s="9" t="s">
         <v>25</v>
@@ -3246,7 +3246,7 @@
         <v>24</v>
       </c>
       <c r="F31" s="9">
-        <v>101</v>
+        <v>82</v>
       </c>
       <c r="G31" s="9" t="s">
         <v>25</v>
@@ -3269,7 +3269,7 @@
         <v>24</v>
       </c>
       <c r="F32" s="9">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="G32" s="9" t="s">
         <v>25</v>
@@ -3292,7 +3292,7 @@
         <v>24</v>
       </c>
       <c r="F33" s="9">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="G33" s="9" t="s">
         <v>25</v>
@@ -3315,7 +3315,7 @@
         <v>24</v>
       </c>
       <c r="F34" s="9">
-        <v>14</v>
+        <v>39</v>
       </c>
       <c r="G34" s="9" t="s">
         <v>25</v>
@@ -3338,7 +3338,7 @@
         <v>24</v>
       </c>
       <c r="F35" s="9">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="G35" s="9" t="s">
         <v>25</v>
@@ -3384,7 +3384,7 @@
         <v>24</v>
       </c>
       <c r="F37" s="9">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G37" s="9" t="s">
         <v>25</v>
@@ -3407,7 +3407,7 @@
         <v>24</v>
       </c>
       <c r="F38" s="9">
-        <v>722</v>
+        <v>739</v>
       </c>
       <c r="G38" s="9" t="s">
         <v>25</v>
@@ -3430,7 +3430,7 @@
         <v>24</v>
       </c>
       <c r="F39" s="9">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="G39" s="9" t="s">
         <v>25</v>
@@ -3453,7 +3453,7 @@
         <v>24</v>
       </c>
       <c r="F40" s="9">
-        <v>784</v>
+        <v>939</v>
       </c>
       <c r="G40" s="9" t="s">
         <v>25</v>
@@ -3476,7 +3476,7 @@
         <v>24</v>
       </c>
       <c r="F41" s="9">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="G41" s="9" t="s">
         <v>25</v>
@@ -3499,7 +3499,7 @@
         <v>24</v>
       </c>
       <c r="F42" s="9">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="G42" s="9" t="s">
         <v>25</v>
@@ -3522,7 +3522,7 @@
         <v>24</v>
       </c>
       <c r="F43" s="9">
-        <v>19</v>
+        <v>52</v>
       </c>
       <c r="G43" s="9" t="s">
         <v>25</v>
@@ -3545,7 +3545,7 @@
         <v>24</v>
       </c>
       <c r="F44" s="9">
-        <v>9</v>
+        <v>33</v>
       </c>
       <c r="G44" s="9" t="s">
         <v>25</v>
@@ -3568,7 +3568,7 @@
         <v>24</v>
       </c>
       <c r="F45" s="9">
-        <v>10</v>
+        <v>29</v>
       </c>
       <c r="G45" s="9" t="s">
         <v>25</v>
@@ -3591,7 +3591,7 @@
         <v>24</v>
       </c>
       <c r="F46" s="9">
-        <v>48</v>
+        <v>100</v>
       </c>
       <c r="G46" s="9" t="s">
         <v>25</v>
@@ -3614,7 +3614,7 @@
         <v>24</v>
       </c>
       <c r="F47" s="9">
-        <v>130</v>
+        <v>143</v>
       </c>
       <c r="G47" s="9" t="s">
         <v>25</v>
@@ -3637,7 +3637,7 @@
         <v>24</v>
       </c>
       <c r="F48" s="9">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="G48" s="9" t="s">
         <v>25</v>
@@ -3660,7 +3660,7 @@
         <v>24</v>
       </c>
       <c r="F49" s="9">
-        <v>2420</v>
+        <v>2493</v>
       </c>
       <c r="G49" s="9" t="s">
         <v>25</v>
@@ -3683,7 +3683,7 @@
         <v>24</v>
       </c>
       <c r="F50" s="9">
-        <v>279</v>
+        <v>387</v>
       </c>
       <c r="G50" s="9" t="s">
         <v>25</v>
@@ -3729,7 +3729,7 @@
         <v>24</v>
       </c>
       <c r="F52" s="9">
-        <v>1732</v>
+        <v>1839</v>
       </c>
       <c r="G52" s="9" t="s">
         <v>25</v>
@@ -3959,7 +3959,7 @@
         <v>24</v>
       </c>
       <c r="F62" s="9">
-        <v>4226</v>
+        <v>4034</v>
       </c>
       <c r="G62" s="9" t="s">
         <v>25</v>
@@ -3982,7 +3982,7 @@
         <v>24</v>
       </c>
       <c r="F63" s="9">
-        <v>3762</v>
+        <v>5294</v>
       </c>
       <c r="G63" s="9" t="s">
         <v>25</v>
@@ -4005,7 +4005,7 @@
         <v>24</v>
       </c>
       <c r="F64" s="9">
-        <v>5335</v>
+        <v>11024</v>
       </c>
       <c r="G64" s="9" t="s">
         <v>25</v>
@@ -4028,7 +4028,7 @@
         <v>24</v>
       </c>
       <c r="F65" s="9">
-        <v>4089</v>
+        <v>6002</v>
       </c>
       <c r="G65" s="9" t="s">
         <v>25</v>
@@ -4051,7 +4051,7 @@
         <v>24</v>
       </c>
       <c r="F66" s="9">
-        <v>5189</v>
+        <v>5774</v>
       </c>
       <c r="G66" s="9" t="s">
         <v>25</v>
@@ -4074,7 +4074,7 @@
         <v>24</v>
       </c>
       <c r="F67" s="9">
-        <v>4614</v>
+        <v>4812</v>
       </c>
       <c r="G67" s="9" t="s">
         <v>25</v>
@@ -4097,7 +4097,7 @@
         <v>24</v>
       </c>
       <c r="F68" s="9">
-        <v>7309</v>
+        <v>7326</v>
       </c>
       <c r="G68" s="9" t="s">
         <v>25</v>
@@ -4120,7 +4120,7 @@
         <v>24</v>
       </c>
       <c r="F69" s="9">
-        <v>2661</v>
+        <v>2672</v>
       </c>
       <c r="G69" s="9" t="s">
         <v>25</v>
@@ -4143,7 +4143,7 @@
         <v>24</v>
       </c>
       <c r="F70" s="9">
-        <v>2916</v>
+        <v>2924</v>
       </c>
       <c r="G70" s="9" t="s">
         <v>25</v>
@@ -4166,7 +4166,7 @@
         <v>24</v>
       </c>
       <c r="F71" s="9">
-        <v>3806</v>
+        <v>4219</v>
       </c>
       <c r="G71" s="9" t="s">
         <v>25</v>
@@ -4189,7 +4189,7 @@
         <v>24</v>
       </c>
       <c r="F72" s="9">
-        <v>3323</v>
+        <v>3593</v>
       </c>
       <c r="G72" s="9" t="s">
         <v>25</v>
@@ -4212,7 +4212,7 @@
         <v>24</v>
       </c>
       <c r="F73" s="9">
-        <v>3461</v>
+        <v>4041</v>
       </c>
       <c r="G73" s="9" t="s">
         <v>25</v>
@@ -4235,7 +4235,7 @@
         <v>24</v>
       </c>
       <c r="F74" s="9">
-        <v>32908</v>
+        <v>34427</v>
       </c>
       <c r="G74" s="9" t="s">
         <v>25</v>
@@ -4258,7 +4258,7 @@
         <v>24</v>
       </c>
       <c r="F75" s="9">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G75" s="9" t="s">
         <v>25</v>
@@ -4327,7 +4327,7 @@
         <v>24</v>
       </c>
       <c r="F78" s="9">
-        <v>1409</v>
+        <v>1364</v>
       </c>
       <c r="G78" s="9" t="s">
         <v>25</v>
@@ -4350,7 +4350,7 @@
         <v>24</v>
       </c>
       <c r="F79" s="9">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G79" s="9" t="s">
         <v>25</v>
@@ -4396,7 +4396,7 @@
         <v>24</v>
       </c>
       <c r="F81" s="9">
-        <v>1116</v>
+        <v>1118</v>
       </c>
       <c r="G81" s="9" t="s">
         <v>25</v>
@@ -4419,7 +4419,7 @@
         <v>24</v>
       </c>
       <c r="F82" s="9">
-        <v>73</v>
+        <v>87</v>
       </c>
       <c r="G82" s="9" t="s">
         <v>25</v>
@@ -4442,7 +4442,7 @@
         <v>24</v>
       </c>
       <c r="F83" s="9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G83" s="9" t="s">
         <v>25</v>
@@ -4465,7 +4465,7 @@
         <v>24</v>
       </c>
       <c r="F84" s="9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G84" s="9" t="s">
         <v>25</v>
@@ -4488,7 +4488,7 @@
         <v>24</v>
       </c>
       <c r="F85" s="9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G85" s="9" t="s">
         <v>25</v>
@@ -4557,7 +4557,7 @@
         <v>24</v>
       </c>
       <c r="F88" s="9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G88" s="9" t="s">
         <v>25</v>
@@ -4626,7 +4626,7 @@
         <v>24</v>
       </c>
       <c r="F91" s="9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G91" s="9" t="s">
         <v>25</v>
@@ -4649,7 +4649,7 @@
         <v>24</v>
       </c>
       <c r="F92" s="9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G92" s="9" t="s">
         <v>25</v>
@@ -4764,7 +4764,7 @@
         <v>24</v>
       </c>
       <c r="F97" s="9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G97" s="9" t="s">
         <v>25</v>
@@ -4787,7 +4787,7 @@
         <v>24</v>
       </c>
       <c r="F98" s="9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G98" s="9" t="s">
         <v>25</v>
@@ -4948,7 +4948,7 @@
         <v>24</v>
       </c>
       <c r="F105" s="9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G105" s="9" t="s">
         <v>25</v>
@@ -4994,7 +4994,7 @@
         <v>24</v>
       </c>
       <c r="F107" s="9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G107" s="9" t="s">
         <v>25</v>
@@ -5017,7 +5017,7 @@
         <v>24</v>
       </c>
       <c r="F108" s="9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G108" s="9" t="s">
         <v>25</v>
@@ -5086,7 +5086,7 @@
         <v>24</v>
       </c>
       <c r="F111" s="9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G111" s="9" t="s">
         <v>25</v>
@@ -5155,7 +5155,7 @@
         <v>24</v>
       </c>
       <c r="F114" s="9">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G114" s="9" t="s">
         <v>25</v>
@@ -5178,7 +5178,7 @@
         <v>24</v>
       </c>
       <c r="F115" s="9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G115" s="9" t="s">
         <v>25</v>
@@ -5270,7 +5270,7 @@
         <v>24</v>
       </c>
       <c r="F119" s="9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G119" s="9" t="s">
         <v>25</v>
@@ -5477,7 +5477,7 @@
         <v>24</v>
       </c>
       <c r="F128" s="9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G128" s="9" t="s">
         <v>25</v>
@@ -5661,7 +5661,7 @@
         <v>24</v>
       </c>
       <c r="F136" s="9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G136" s="9" t="s">
         <v>25</v>
@@ -5937,7 +5937,7 @@
         <v>24</v>
       </c>
       <c r="F148" s="9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G148" s="9" t="s">
         <v>25</v>
@@ -6006,7 +6006,7 @@
         <v>24</v>
       </c>
       <c r="F151" s="9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G151" s="9" t="s">
         <v>25</v>
@@ -6052,7 +6052,7 @@
         <v>24</v>
       </c>
       <c r="F153" s="9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G153" s="9" t="s">
         <v>25</v>
@@ -6075,7 +6075,7 @@
         <v>24</v>
       </c>
       <c r="F154" s="9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G154" s="9" t="s">
         <v>25</v>
@@ -6098,7 +6098,7 @@
         <v>24</v>
       </c>
       <c r="F155" s="9">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G155" s="9" t="s">
         <v>25</v>
@@ -6213,7 +6213,7 @@
         <v>24</v>
       </c>
       <c r="F160" s="9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G160" s="9" t="s">
         <v>25</v>
@@ -6259,7 +6259,7 @@
         <v>24</v>
       </c>
       <c r="F162" s="9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G162" s="9" t="s">
         <v>25</v>
@@ -6512,7 +6512,7 @@
         <v>24</v>
       </c>
       <c r="F173" s="9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G173" s="9" t="s">
         <v>25</v>
@@ -6604,7 +6604,7 @@
         <v>24</v>
       </c>
       <c r="F177" s="9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G177" s="9" t="s">
         <v>25</v>
@@ -6903,7 +6903,7 @@
         <v>24</v>
       </c>
       <c r="F190" s="9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G190" s="9" t="s">
         <v>25</v>
@@ -7018,7 +7018,7 @@
         <v>24</v>
       </c>
       <c r="F195" s="9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G195" s="9" t="s">
         <v>25</v>
@@ -7110,7 +7110,7 @@
         <v>24</v>
       </c>
       <c r="F199" s="9">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="G199" s="9" t="s">
         <v>25</v>
@@ -7179,7 +7179,7 @@
         <v>24</v>
       </c>
       <c r="F202" s="9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G202" s="9" t="s">
         <v>25</v>
@@ -7202,7 +7202,7 @@
         <v>24</v>
       </c>
       <c r="F203" s="9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G203" s="9" t="s">
         <v>25</v>

</xml_diff>

<commit_message>
chore: optimize appium test runner and configure GHA to run on ubuntu-latest
</commit_message>
<xml_diff>
--- a/selenium-tests/test-report.xlsx
+++ b/selenium-tests/test-report.xlsx
@@ -21,13 +21,13 @@
     <t>Report Date:</t>
   </si>
   <si>
-    <t>22/6/2026, 11:38:17 am</t>
+    <t>22/6/2026, 3:28:30 pm</t>
   </si>
   <si>
     <t>Total Duration:</t>
   </si>
   <si>
-    <t>129.43 seconds</t>
+    <t>128.98 seconds</t>
   </si>
   <si>
     <t/>
@@ -2579,7 +2579,7 @@
         <v>24</v>
       </c>
       <c r="F2" s="9">
-        <v>5044</v>
+        <v>4592</v>
       </c>
       <c r="G2" s="9" t="s">
         <v>25</v>
@@ -2602,7 +2602,7 @@
         <v>24</v>
       </c>
       <c r="F3" s="9">
-        <v>2569</v>
+        <v>2014</v>
       </c>
       <c r="G3" s="9" t="s">
         <v>25</v>
@@ -2625,7 +2625,7 @@
         <v>24</v>
       </c>
       <c r="F4" s="9">
-        <v>1482</v>
+        <v>2003</v>
       </c>
       <c r="G4" s="9" t="s">
         <v>25</v>
@@ -2648,7 +2648,7 @@
         <v>24</v>
       </c>
       <c r="F5" s="9">
-        <v>301</v>
+        <v>338</v>
       </c>
       <c r="G5" s="9" t="s">
         <v>25</v>
@@ -2671,7 +2671,7 @@
         <v>24</v>
       </c>
       <c r="F6" s="9">
-        <v>863</v>
+        <v>952</v>
       </c>
       <c r="G6" s="9" t="s">
         <v>25</v>
@@ -2694,7 +2694,7 @@
         <v>24</v>
       </c>
       <c r="F7" s="9">
-        <v>775</v>
+        <v>797</v>
       </c>
       <c r="G7" s="9" t="s">
         <v>25</v>
@@ -2717,7 +2717,7 @@
         <v>24</v>
       </c>
       <c r="F8" s="9">
-        <v>29</v>
+        <v>41</v>
       </c>
       <c r="G8" s="9" t="s">
         <v>25</v>
@@ -2740,7 +2740,7 @@
         <v>24</v>
       </c>
       <c r="F9" s="9">
-        <v>8</v>
+        <v>19</v>
       </c>
       <c r="G9" s="9" t="s">
         <v>25</v>
@@ -2763,7 +2763,7 @@
         <v>24</v>
       </c>
       <c r="F10" s="9">
-        <v>17</v>
+        <v>33</v>
       </c>
       <c r="G10" s="9" t="s">
         <v>25</v>
@@ -2786,7 +2786,7 @@
         <v>24</v>
       </c>
       <c r="F11" s="9">
-        <v>22</v>
+        <v>42</v>
       </c>
       <c r="G11" s="9" t="s">
         <v>25</v>
@@ -2809,7 +2809,7 @@
         <v>24</v>
       </c>
       <c r="F12" s="9">
-        <v>772</v>
+        <v>782</v>
       </c>
       <c r="G12" s="9" t="s">
         <v>25</v>
@@ -2832,7 +2832,7 @@
         <v>24</v>
       </c>
       <c r="F13" s="9">
-        <v>201</v>
+        <v>246</v>
       </c>
       <c r="G13" s="9" t="s">
         <v>25</v>
@@ -2855,7 +2855,7 @@
         <v>24</v>
       </c>
       <c r="F14" s="9">
-        <v>927</v>
+        <v>834</v>
       </c>
       <c r="G14" s="9" t="s">
         <v>25</v>
@@ -2878,7 +2878,7 @@
         <v>24</v>
       </c>
       <c r="F15" s="9">
-        <v>981</v>
+        <v>1028</v>
       </c>
       <c r="G15" s="9" t="s">
         <v>25</v>
@@ -2901,7 +2901,7 @@
         <v>24</v>
       </c>
       <c r="F16" s="9">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="G16" s="9" t="s">
         <v>25</v>
@@ -2924,7 +2924,7 @@
         <v>24</v>
       </c>
       <c r="F17" s="9">
-        <v>114</v>
+        <v>96</v>
       </c>
       <c r="G17" s="9" t="s">
         <v>25</v>
@@ -2947,7 +2947,7 @@
         <v>24</v>
       </c>
       <c r="F18" s="9">
-        <v>461</v>
+        <v>485</v>
       </c>
       <c r="G18" s="9" t="s">
         <v>25</v>
@@ -2970,7 +2970,7 @@
         <v>24</v>
       </c>
       <c r="F19" s="9">
-        <v>568</v>
+        <v>522</v>
       </c>
       <c r="G19" s="9" t="s">
         <v>25</v>
@@ -2993,7 +2993,7 @@
         <v>24</v>
       </c>
       <c r="F20" s="9">
-        <v>397</v>
+        <v>171</v>
       </c>
       <c r="G20" s="9" t="s">
         <v>25</v>
@@ -3016,7 +3016,7 @@
         <v>24</v>
       </c>
       <c r="F21" s="9">
-        <v>1259</v>
+        <v>797</v>
       </c>
       <c r="G21" s="9" t="s">
         <v>25</v>
@@ -3039,7 +3039,7 @@
         <v>24</v>
       </c>
       <c r="F22" s="9">
-        <v>954</v>
+        <v>778</v>
       </c>
       <c r="G22" s="9" t="s">
         <v>25</v>
@@ -3062,7 +3062,7 @@
         <v>24</v>
       </c>
       <c r="F23" s="9">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="G23" s="9" t="s">
         <v>25</v>
@@ -3085,7 +3085,7 @@
         <v>24</v>
       </c>
       <c r="F24" s="9">
-        <v>112</v>
+        <v>92</v>
       </c>
       <c r="G24" s="9" t="s">
         <v>25</v>
@@ -3108,7 +3108,7 @@
         <v>24</v>
       </c>
       <c r="F25" s="9">
-        <v>448</v>
+        <v>438</v>
       </c>
       <c r="G25" s="9" t="s">
         <v>25</v>
@@ -3131,7 +3131,7 @@
         <v>24</v>
       </c>
       <c r="F26" s="9">
-        <v>775</v>
+        <v>768</v>
       </c>
       <c r="G26" s="9" t="s">
         <v>25</v>
@@ -3154,7 +3154,7 @@
         <v>24</v>
       </c>
       <c r="F27" s="9">
-        <v>1243</v>
+        <v>1294</v>
       </c>
       <c r="G27" s="9" t="s">
         <v>25</v>
@@ -3177,7 +3177,7 @@
         <v>24</v>
       </c>
       <c r="F28" s="9">
-        <v>1213</v>
+        <v>1254</v>
       </c>
       <c r="G28" s="9" t="s">
         <v>25</v>
@@ -3200,7 +3200,7 @@
         <v>24</v>
       </c>
       <c r="F29" s="9">
-        <v>1195</v>
+        <v>1225</v>
       </c>
       <c r="G29" s="9" t="s">
         <v>25</v>
@@ -3223,7 +3223,7 @@
         <v>24</v>
       </c>
       <c r="F30" s="9">
-        <v>768</v>
+        <v>879</v>
       </c>
       <c r="G30" s="9" t="s">
         <v>25</v>
@@ -3246,7 +3246,7 @@
         <v>24</v>
       </c>
       <c r="F31" s="9">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="G31" s="9" t="s">
         <v>25</v>
@@ -3269,7 +3269,7 @@
         <v>24</v>
       </c>
       <c r="F32" s="9">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="G32" s="9" t="s">
         <v>25</v>
@@ -3292,7 +3292,7 @@
         <v>24</v>
       </c>
       <c r="F33" s="9">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="G33" s="9" t="s">
         <v>25</v>
@@ -3315,7 +3315,7 @@
         <v>24</v>
       </c>
       <c r="F34" s="9">
-        <v>39</v>
+        <v>16</v>
       </c>
       <c r="G34" s="9" t="s">
         <v>25</v>
@@ -3338,7 +3338,7 @@
         <v>24</v>
       </c>
       <c r="F35" s="9">
-        <v>30</v>
+        <v>59</v>
       </c>
       <c r="G35" s="9" t="s">
         <v>25</v>
@@ -3361,7 +3361,7 @@
         <v>24</v>
       </c>
       <c r="F36" s="9">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="G36" s="9" t="s">
         <v>25</v>
@@ -3384,7 +3384,7 @@
         <v>24</v>
       </c>
       <c r="F37" s="9">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="G37" s="9" t="s">
         <v>25</v>
@@ -3407,7 +3407,7 @@
         <v>24</v>
       </c>
       <c r="F38" s="9">
-        <v>739</v>
+        <v>749</v>
       </c>
       <c r="G38" s="9" t="s">
         <v>25</v>
@@ -3430,7 +3430,7 @@
         <v>24</v>
       </c>
       <c r="F39" s="9">
-        <v>30</v>
+        <v>12</v>
       </c>
       <c r="G39" s="9" t="s">
         <v>25</v>
@@ -3453,7 +3453,7 @@
         <v>24</v>
       </c>
       <c r="F40" s="9">
-        <v>939</v>
+        <v>789</v>
       </c>
       <c r="G40" s="9" t="s">
         <v>25</v>
@@ -3476,7 +3476,7 @@
         <v>24</v>
       </c>
       <c r="F41" s="9">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="G41" s="9" t="s">
         <v>25</v>
@@ -3499,7 +3499,7 @@
         <v>24</v>
       </c>
       <c r="F42" s="9">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G42" s="9" t="s">
         <v>25</v>
@@ -3522,7 +3522,7 @@
         <v>24</v>
       </c>
       <c r="F43" s="9">
-        <v>52</v>
+        <v>18</v>
       </c>
       <c r="G43" s="9" t="s">
         <v>25</v>
@@ -3545,7 +3545,7 @@
         <v>24</v>
       </c>
       <c r="F44" s="9">
-        <v>33</v>
+        <v>10</v>
       </c>
       <c r="G44" s="9" t="s">
         <v>25</v>
@@ -3568,7 +3568,7 @@
         <v>24</v>
       </c>
       <c r="F45" s="9">
-        <v>29</v>
+        <v>10</v>
       </c>
       <c r="G45" s="9" t="s">
         <v>25</v>
@@ -3591,7 +3591,7 @@
         <v>24</v>
       </c>
       <c r="F46" s="9">
-        <v>100</v>
+        <v>32</v>
       </c>
       <c r="G46" s="9" t="s">
         <v>25</v>
@@ -3614,7 +3614,7 @@
         <v>24</v>
       </c>
       <c r="F47" s="9">
-        <v>143</v>
+        <v>118</v>
       </c>
       <c r="G47" s="9" t="s">
         <v>25</v>
@@ -3637,7 +3637,7 @@
         <v>24</v>
       </c>
       <c r="F48" s="9">
-        <v>82</v>
+        <v>66</v>
       </c>
       <c r="G48" s="9" t="s">
         <v>25</v>
@@ -3660,7 +3660,7 @@
         <v>24</v>
       </c>
       <c r="F49" s="9">
-        <v>2493</v>
+        <v>2366</v>
       </c>
       <c r="G49" s="9" t="s">
         <v>25</v>
@@ -3683,7 +3683,7 @@
         <v>24</v>
       </c>
       <c r="F50" s="9">
-        <v>387</v>
+        <v>333</v>
       </c>
       <c r="G50" s="9" t="s">
         <v>25</v>
@@ -3729,7 +3729,7 @@
         <v>24</v>
       </c>
       <c r="F52" s="9">
-        <v>1839</v>
+        <v>1772</v>
       </c>
       <c r="G52" s="9" t="s">
         <v>25</v>
@@ -3959,7 +3959,7 @@
         <v>24</v>
       </c>
       <c r="F62" s="9">
-        <v>4034</v>
+        <v>4544</v>
       </c>
       <c r="G62" s="9" t="s">
         <v>25</v>
@@ -3982,7 +3982,7 @@
         <v>24</v>
       </c>
       <c r="F63" s="9">
-        <v>5294</v>
+        <v>5016</v>
       </c>
       <c r="G63" s="9" t="s">
         <v>25</v>
@@ -4005,7 +4005,7 @@
         <v>24</v>
       </c>
       <c r="F64" s="9">
-        <v>11024</v>
+        <v>6061</v>
       </c>
       <c r="G64" s="9" t="s">
         <v>25</v>
@@ -4028,7 +4028,7 @@
         <v>24</v>
       </c>
       <c r="F65" s="9">
-        <v>6002</v>
+        <v>4259</v>
       </c>
       <c r="G65" s="9" t="s">
         <v>25</v>
@@ -4051,7 +4051,7 @@
         <v>24</v>
       </c>
       <c r="F66" s="9">
-        <v>5774</v>
+        <v>5606</v>
       </c>
       <c r="G66" s="9" t="s">
         <v>25</v>
@@ -4074,7 +4074,7 @@
         <v>24</v>
       </c>
       <c r="F67" s="9">
-        <v>4812</v>
+        <v>4832</v>
       </c>
       <c r="G67" s="9" t="s">
         <v>25</v>
@@ -4097,7 +4097,7 @@
         <v>24</v>
       </c>
       <c r="F68" s="9">
-        <v>7326</v>
+        <v>8134</v>
       </c>
       <c r="G68" s="9" t="s">
         <v>25</v>
@@ -4120,7 +4120,7 @@
         <v>24</v>
       </c>
       <c r="F69" s="9">
-        <v>2672</v>
+        <v>2755</v>
       </c>
       <c r="G69" s="9" t="s">
         <v>25</v>
@@ -4143,7 +4143,7 @@
         <v>24</v>
       </c>
       <c r="F70" s="9">
-        <v>2924</v>
+        <v>3005</v>
       </c>
       <c r="G70" s="9" t="s">
         <v>25</v>
@@ -4166,7 +4166,7 @@
         <v>24</v>
       </c>
       <c r="F71" s="9">
-        <v>4219</v>
+        <v>4118</v>
       </c>
       <c r="G71" s="9" t="s">
         <v>25</v>
@@ -4189,7 +4189,7 @@
         <v>24</v>
       </c>
       <c r="F72" s="9">
-        <v>3593</v>
+        <v>3504</v>
       </c>
       <c r="G72" s="9" t="s">
         <v>25</v>
@@ -4212,7 +4212,7 @@
         <v>24</v>
       </c>
       <c r="F73" s="9">
-        <v>4041</v>
+        <v>4429</v>
       </c>
       <c r="G73" s="9" t="s">
         <v>25</v>
@@ -4235,7 +4235,7 @@
         <v>24</v>
       </c>
       <c r="F74" s="9">
-        <v>34427</v>
+        <v>40759</v>
       </c>
       <c r="G74" s="9" t="s">
         <v>25</v>
@@ -4258,7 +4258,7 @@
         <v>24</v>
       </c>
       <c r="F75" s="9">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="G75" s="9" t="s">
         <v>25</v>
@@ -4327,7 +4327,7 @@
         <v>24</v>
       </c>
       <c r="F78" s="9">
-        <v>1364</v>
+        <v>1550</v>
       </c>
       <c r="G78" s="9" t="s">
         <v>25</v>
@@ -4350,7 +4350,7 @@
         <v>24</v>
       </c>
       <c r="F79" s="9">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G79" s="9" t="s">
         <v>25</v>
@@ -4396,7 +4396,7 @@
         <v>24</v>
       </c>
       <c r="F81" s="9">
-        <v>1118</v>
+        <v>1194</v>
       </c>
       <c r="G81" s="9" t="s">
         <v>25</v>
@@ -4419,7 +4419,7 @@
         <v>24</v>
       </c>
       <c r="F82" s="9">
-        <v>87</v>
+        <v>113</v>
       </c>
       <c r="G82" s="9" t="s">
         <v>25</v>
@@ -4465,7 +4465,7 @@
         <v>24</v>
       </c>
       <c r="F84" s="9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G84" s="9" t="s">
         <v>25</v>
@@ -4534,7 +4534,7 @@
         <v>24</v>
       </c>
       <c r="F87" s="9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G87" s="9" t="s">
         <v>25</v>
@@ -4557,7 +4557,7 @@
         <v>24</v>
       </c>
       <c r="F88" s="9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G88" s="9" t="s">
         <v>25</v>
@@ -4626,7 +4626,7 @@
         <v>24</v>
       </c>
       <c r="F91" s="9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G91" s="9" t="s">
         <v>25</v>
@@ -4764,7 +4764,7 @@
         <v>24</v>
       </c>
       <c r="F97" s="9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G97" s="9" t="s">
         <v>25</v>
@@ -4787,7 +4787,7 @@
         <v>24</v>
       </c>
       <c r="F98" s="9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G98" s="9" t="s">
         <v>25</v>
@@ -4810,7 +4810,7 @@
         <v>24</v>
       </c>
       <c r="F99" s="9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G99" s="9" t="s">
         <v>25</v>
@@ -4948,7 +4948,7 @@
         <v>24</v>
       </c>
       <c r="F105" s="9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G105" s="9" t="s">
         <v>25</v>
@@ -4994,7 +4994,7 @@
         <v>24</v>
       </c>
       <c r="F107" s="9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G107" s="9" t="s">
         <v>25</v>
@@ -5017,7 +5017,7 @@
         <v>24</v>
       </c>
       <c r="F108" s="9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G108" s="9" t="s">
         <v>25</v>
@@ -5086,7 +5086,7 @@
         <v>24</v>
       </c>
       <c r="F111" s="9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G111" s="9" t="s">
         <v>25</v>
@@ -5132,7 +5132,7 @@
         <v>24</v>
       </c>
       <c r="F113" s="9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G113" s="9" t="s">
         <v>25</v>
@@ -5155,7 +5155,7 @@
         <v>24</v>
       </c>
       <c r="F114" s="9">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G114" s="9" t="s">
         <v>25</v>
@@ -5178,7 +5178,7 @@
         <v>24</v>
       </c>
       <c r="F115" s="9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G115" s="9" t="s">
         <v>25</v>
@@ -5270,7 +5270,7 @@
         <v>24</v>
       </c>
       <c r="F119" s="9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G119" s="9" t="s">
         <v>25</v>
@@ -5408,7 +5408,7 @@
         <v>24</v>
       </c>
       <c r="F125" s="9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G125" s="9" t="s">
         <v>25</v>
@@ -5661,7 +5661,7 @@
         <v>24</v>
       </c>
       <c r="F136" s="9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G136" s="9" t="s">
         <v>25</v>
@@ -5845,7 +5845,7 @@
         <v>24</v>
       </c>
       <c r="F144" s="9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G144" s="9" t="s">
         <v>25</v>
@@ -5937,7 +5937,7 @@
         <v>24</v>
       </c>
       <c r="F148" s="9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G148" s="9" t="s">
         <v>25</v>
@@ -6006,7 +6006,7 @@
         <v>24</v>
       </c>
       <c r="F151" s="9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G151" s="9" t="s">
         <v>25</v>
@@ -6052,7 +6052,7 @@
         <v>24</v>
       </c>
       <c r="F153" s="9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G153" s="9" t="s">
         <v>25</v>
@@ -6098,7 +6098,7 @@
         <v>24</v>
       </c>
       <c r="F155" s="9">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="G155" s="9" t="s">
         <v>25</v>
@@ -6121,7 +6121,7 @@
         <v>24</v>
       </c>
       <c r="F156" s="9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G156" s="9" t="s">
         <v>25</v>
@@ -6213,7 +6213,7 @@
         <v>24</v>
       </c>
       <c r="F160" s="9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G160" s="9" t="s">
         <v>25</v>
@@ -6259,7 +6259,7 @@
         <v>24</v>
       </c>
       <c r="F162" s="9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G162" s="9" t="s">
         <v>25</v>
@@ -6420,7 +6420,7 @@
         <v>24</v>
       </c>
       <c r="F169" s="9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G169" s="9" t="s">
         <v>25</v>
@@ -6604,7 +6604,7 @@
         <v>24</v>
       </c>
       <c r="F177" s="9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G177" s="9" t="s">
         <v>25</v>
@@ -6903,7 +6903,7 @@
         <v>24</v>
       </c>
       <c r="F190" s="9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G190" s="9" t="s">
         <v>25</v>
@@ -7110,7 +7110,7 @@
         <v>24</v>
       </c>
       <c r="F199" s="9">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="G199" s="9" t="s">
         <v>25</v>
@@ -7179,7 +7179,7 @@
         <v>24</v>
       </c>
       <c r="F202" s="9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G202" s="9" t="s">
         <v>25</v>
@@ -7202,7 +7202,7 @@
         <v>24</v>
       </c>
       <c r="F203" s="9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G203" s="9" t="s">
         <v>25</v>

</xml_diff>